<commit_message>
added a new ai analyser
</commit_message>
<xml_diff>
--- a/KeywordsResponses.xlsx
+++ b/KeywordsResponses.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\divya\OneDrive\Documents\Kavish's Documents\UIPATHING\AutoEmailResponder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kav's Downloads\UIPATHING\MailAutoResponder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F140A699-A20E-4217-A742-A87BB3F81A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5801175C-FEF5-40C8-B3A8-92FD3367E77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2544" yWindow="4836" windowWidth="19656" windowHeight="10932" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5655" yWindow="1485" windowWidth="21810" windowHeight="12960" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -401,12 +401,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="64.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -414,7 +414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -422,7 +422,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -430,7 +430,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -446,9 +446,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{497D2ACF-05DF-4692-B6DB-91A48E9CC310}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -461,9 +461,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC6FB1A-4F3C-4104-BB5F-87C609F81CD0}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -475,14 +475,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D710969B-ACF5-4DB1-BCAD-E16B23DDD428}">
-  <dimension ref="B1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
       <c r="B1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
All features working, Check emails address
</commit_message>
<xml_diff>
--- a/KeywordsResponses.xlsx
+++ b/KeywordsResponses.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kav's Downloads\UIPATHING\MailAutoResponder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5801175C-FEF5-40C8-B3A8-92FD3367E77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F3666A-4826-4FFC-8DD0-85715666892A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5655" yWindow="1485" windowWidth="21810" windowHeight="12960" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5655" yWindow="1485" windowWidth="21810" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,14 +28,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
   <si>
     <t>Keyword</t>
   </si>
   <si>
-    <t>Response</t>
-  </si>
-  <si>
     <t>Password</t>
   </si>
   <si>
@@ -45,26 +42,170 @@
     <t>VPN</t>
   </si>
   <si>
-    <t>Please reset your password via the self-service portal at reset.company.com.</t>
-  </si>
-  <si>
-    <t>Please restart your VPN client and reconnect. If the issue persists, contact IT.</t>
-  </si>
-  <si>
-    <t>Please check the printer is powered on and connected to the network.</t>
-  </si>
-  <si>
     <t>Department</t>
   </si>
   <si>
     <t>Email</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Account</t>
+  </si>
+  <si>
+    <t>Report</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Leave</t>
+  </si>
+  <si>
+    <t>Meeting</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Server</t>
+  </si>
+  <si>
+    <t>Access</t>
+  </si>
+  <si>
+    <t>Outlook</t>
+  </si>
+  <si>
+    <t>Software</t>
+  </si>
+  <si>
+    <t>Network</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Internet</t>
+  </si>
+  <si>
+    <t>advertisement</t>
+  </si>
+  <si>
+    <t>promotion</t>
+  </si>
+  <si>
+    <t>discount</t>
+  </si>
+  <si>
+    <t>offer</t>
+  </si>
+  <si>
+    <t>winner</t>
+  </si>
+  <si>
+    <t>prize</t>
+  </si>
+  <si>
+    <t>free</t>
+  </si>
+  <si>
+    <t>casino</t>
+  </si>
+  <si>
+    <t>lottery</t>
+  </si>
+  <si>
+    <t>investment</t>
+  </si>
+  <si>
+    <t>crypto</t>
+  </si>
+  <si>
+    <t>bitcoin</t>
+  </si>
+  <si>
+    <t>loan</t>
+  </si>
+  <si>
+    <t>marketing</t>
+  </si>
+  <si>
+    <t>unsubscribe</t>
+  </si>
+  <si>
+    <t>urgent</t>
+  </si>
+  <si>
+    <t>emergency</t>
+  </si>
+  <si>
+    <t>critical</t>
+  </si>
+  <si>
+    <t>immediately</t>
+  </si>
+  <si>
+    <t>asap</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>important</t>
+  </si>
+  <si>
+    <t>alert</t>
+  </si>
+  <si>
+    <t>failure</t>
+  </si>
+  <si>
+    <t>outage</t>
+  </si>
+  <si>
+    <t>down</t>
+  </si>
+  <si>
+    <t>blocked</t>
+  </si>
+  <si>
+    <t>security</t>
+  </si>
+  <si>
+    <t>breach</t>
+  </si>
+  <si>
+    <t>deadline</t>
+  </si>
+  <si>
+    <t>IT Department</t>
+  </si>
+  <si>
+    <t>Finance Department</t>
+  </si>
+  <si>
+    <t>HR Department</t>
+  </si>
+  <si>
+    <t>klimovgag@gmail.com</t>
+  </si>
+  <si>
+    <t>General</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +217,19 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -113,15 +267,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -400,42 +561,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="64.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="3" spans="1:1">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -445,12 +679,87 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{497D2ACF-05DF-4692-B6DB-91A48E9CC310}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="3" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -460,12 +769,87 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC6FB1A-4F3C-4104-BB5F-87C609F81CD0}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -475,18 +859,56 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D710969B-ACF5-4DB1-BCAD-E16B23DDD428}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{D8F2E156-1F93-42B8-B692-F8DCF44AB446}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{772FE154-83CC-475C-96F7-2F8A4C863011}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{4BBEFB24-57CA-4787-A9B0-AAE2E490AE92}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{C8B6B913-22A8-4824-B200-5FE4254DEA06}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>